<commit_message>
reconstruct the skills using double invoking method, to ensure the costs and text-information of skills are called whenever you evoke a skill; the effects are now playing in rows, VFX is abandoned, EffectManager now takes over; Buffs are now added into our system; Sword and AvailbleSword are now merged as one Observable; A CheatManager is added for convenience, New levels are added; the skills of heroes are disabled temporarily
</commit_message>
<xml_diff>
--- a/Src/Assets/StreamingAssets/Common/Tables/Tables/Versus.xlsx
+++ b/Src/Assets/StreamingAssets/Common/Tables/Tables/Versus.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CCA\Src\Assets\Common\Tables\Tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CCA\Src\Assets\StreamingAssets\Common\Tables\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D4C9FB-E2F9-4A80-8B29-B73B7927668A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF5AB051-4D76-439D-A791-D5C03C76BA8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attack_Defend_Counter_2dArray" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -146,11 +146,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -164,7 +164,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -568,17 +568,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I15"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24.33203125" customWidth="1"/>
-    <col min="3" max="3" width="16.58203125" customWidth="1"/>
-    <col min="4" max="4" width="12.08203125" customWidth="1"/>
-    <col min="5" max="5" width="13.75" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" customWidth="1"/>
-    <col min="9" max="9" width="14.25" customWidth="1"/>
+    <col min="1" max="1" width="24.36328125" customWidth="1"/>
+    <col min="3" max="3" width="16.54296875" customWidth="1"/>
+    <col min="4" max="4" width="12.08984375" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" customWidth="1"/>
+    <col min="7" max="7" width="10.6328125" customWidth="1"/>
+    <col min="9" max="9" width="14.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -607,7 +607,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="15">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -636,7 +636,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="15">
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
@@ -665,7 +665,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="15">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -694,7 +694,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="15">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -723,7 +723,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="15">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -752,7 +752,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="15">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -781,7 +781,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="15">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -810,7 +810,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="15">
       <c r="A9" s="6" t="s">
         <v>7</v>
       </c>
@@ -839,7 +839,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="15">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -868,7 +868,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="15">
       <c r="A11" s="6" t="s">
         <v>23</v>
       </c>
@@ -897,7 +897,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="15">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
@@ -926,7 +926,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="15">
       <c r="A13" s="6" t="s">
         <v>10</v>
       </c>
@@ -955,7 +955,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="15">
       <c r="A14" s="3" t="s">
         <v>25</v>
       </c>
@@ -984,7 +984,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="15">
       <c r="A15" s="13" t="s">
         <v>26</v>
       </c>

</xml_diff>